<commit_message>
style(vehicle-export): bold the row-1 title in all category templates
Turned the row-1 title bold (kept Bernard MT Condensed 26pt) across all five
templates' sheets. Since export fills these templates, the bold title shows on
both the template download and the filled export.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Pelawat.xlsx
+++ b/assets/templates/Pelawat.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="3" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView activeTab="11" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="JANUARI" sheetId="1" r:id="rId4"/>
@@ -96,7 +96,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -119,6 +119,15 @@
     </font>
     <font>
       <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Bernard MT Condensed"/>
+    </font>
+    <font>
+      <b val="1"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
@@ -258,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -319,6 +328,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="9" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -668,7 +683,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="19"/>
@@ -1293,7 +1308,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="20"/>
@@ -1919,7 +1934,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>19</v>
       </c>
       <c r="B1" s="20"/>
@@ -2543,7 +2558,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="20"/>
@@ -3166,7 +3181,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="19"/>
@@ -3789,7 +3804,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="19"/>
@@ -4412,7 +4427,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="19"/>
@@ -5035,7 +5050,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="19"/>
@@ -5658,7 +5673,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="19"/>
@@ -6281,7 +6296,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="20"/>
@@ -6904,7 +6919,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="20"/>
@@ -7529,7 +7544,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>17</v>
       </c>
       <c r="B1" s="20"/>

</xml_diff>

<commit_message>
revert: keep row-1 title not-bold to match the official form exactly
The official Polis Bantuan forms use Bernard MT Condensed 26pt, NOT bold, for
the row-1 title (verified across all four forms). The earlier bold edit was the
only thing making the template/export differ from the form, so revert it. Row 1
now matches the official form byte-for-byte (the four official templates are
restored to their pristine files; Pelawat stays its Staf-derived copy).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Pelawat.xlsx
+++ b/assets/templates/Pelawat.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="11" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView activeTab="3" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="JANUARI" sheetId="1" r:id="rId4"/>
@@ -96,7 +96,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -119,15 +119,6 @@
     </font>
     <font>
       <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="26"/>
-      <color theme="1"/>
-      <name val="Bernard MT Condensed"/>
-    </font>
-    <font>
-      <b val="1"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
@@ -267,7 +258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -328,12 +319,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="9" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,7 +668,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="19"/>
@@ -1308,7 +1293,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="20"/>
@@ -1934,7 +1919,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>19</v>
       </c>
       <c r="B1" s="20"/>
@@ -2558,7 +2543,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="20"/>
@@ -3181,7 +3166,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="19"/>
@@ -3804,7 +3789,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="19"/>
@@ -4427,7 +4412,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="19"/>
@@ -5050,7 +5035,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="19"/>
@@ -5673,7 +5658,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="19"/>
@@ -6296,7 +6281,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="20"/>
@@ -6919,7 +6904,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="20"/>
@@ -7544,7 +7529,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B1" s="20"/>

</xml_diff>

<commit_message>
style(vehicle-export): bold the row-1 title per user preference
User prefers a bold title (heavier than the official form, which is not bold).
Set A1 bold across all sheets of all five templates; since export fills these
templates, both the template download and the filled export show the bold title
and stay identical.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Pelawat.xlsx
+++ b/assets/templates/Pelawat.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="3" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView activeTab="11" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="JANUARI" sheetId="1" r:id="rId4"/>
@@ -96,7 +96,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -119,6 +119,15 @@
     </font>
     <font>
       <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Bernard MT Condensed"/>
+    </font>
+    <font>
+      <b val="1"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
@@ -258,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -319,6 +328,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="9" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -668,7 +683,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="19"/>
@@ -1293,7 +1308,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="20"/>
@@ -1919,7 +1934,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>19</v>
       </c>
       <c r="B1" s="20"/>
@@ -2543,7 +2558,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="20"/>
@@ -3166,7 +3181,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="19"/>
@@ -3789,7 +3804,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="19"/>
@@ -4412,7 +4427,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="19"/>
@@ -5035,7 +5050,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="19"/>
@@ -5658,7 +5673,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="19"/>
@@ -6281,7 +6296,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="20"/>
@@ -6904,7 +6919,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="20"/>
@@ -7529,7 +7544,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customHeight="1" ht="32.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="23" t="s">
         <v>17</v>
       </c>
       <c r="B1" s="20"/>

</xml_diff>

<commit_message>
revert: row-1 title not-bold to exactly match the original form
Per user: the template/export must be exactly like the original official form,
which is NOT bold. Restore the not-bold templates so row 1 matches the form
byte-for-byte. Export fills these, so it matches too.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Pelawat.xlsx
+++ b/assets/templates/Pelawat.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="11" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView activeTab="3" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="JANUARI" sheetId="1" r:id="rId4"/>
@@ -96,7 +96,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -119,15 +119,6 @@
     </font>
     <font>
       <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="26"/>
-      <color theme="1"/>
-      <name val="Bernard MT Condensed"/>
-    </font>
-    <font>
-      <b val="1"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
@@ -267,7 +258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -328,12 +319,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="9" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,7 +668,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="19"/>
@@ -1308,7 +1293,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="20"/>
@@ -1934,7 +1919,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>19</v>
       </c>
       <c r="B1" s="20"/>
@@ -2558,7 +2543,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="20"/>
@@ -3181,7 +3166,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="19"/>
@@ -3804,7 +3789,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="19"/>
@@ -4427,7 +4412,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="19"/>
@@ -5050,7 +5035,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="19"/>
@@ -5673,7 +5658,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="19"/>
@@ -6296,7 +6281,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="20"/>
@@ -6919,7 +6904,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="20"/>
@@ -7544,7 +7529,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" customHeight="1" ht="32.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B1" s="20"/>

</xml_diff>